<commit_message>
haader en los submodulo de novedades sean modificado para ser mas claros y compactos  .
</commit_message>
<xml_diff>
--- a/sgturnos/mallas/malla_ter04_2026-01.xlsx
+++ b/sgturnos/mallas/malla_ter04_2026-01.xlsx
@@ -517,17 +517,17 @@
       <c r="J3" t="s" s="4">
         <v>40</v>
       </c>
-      <c r="K3" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="L3" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="M3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="N3" t="s" s="5">
-        <v>39</v>
+      <c r="K3" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="L3" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="M3" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="N3" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="O3" t="s" s="2">
         <v>38</v>
@@ -544,17 +544,17 @@
       <c r="S3" t="s" s="4">
         <v>40</v>
       </c>
-      <c r="T3" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="U3" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="V3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="W3" t="s" s="5">
-        <v>39</v>
+      <c r="T3" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="U3" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="V3" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="W3" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="X3" t="s" s="2">
         <v>38</v>
@@ -571,17 +571,17 @@
       <c r="AB3" t="s" s="4">
         <v>40</v>
       </c>
-      <c r="AC3" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="AD3" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="AE3" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AF3" t="s" s="5">
-        <v>39</v>
+      <c r="AC3" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="AD3" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="AE3" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="AF3" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="AG3" t="s" s="0">
         <v>41</v>
@@ -600,32 +600,32 @@
       <c r="C4" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="D4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="E4" t="s" s="5">
-        <v>39</v>
-      </c>
-      <c r="F4" t="s" s="6">
+      <c r="D4" t="s" s="6">
         <v>36</v>
       </c>
+      <c r="E4" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s" s="3">
+        <v>37</v>
+      </c>
       <c r="G4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="H4" t="s" s="3">
-        <v>37</v>
+      <c r="H4" t="s" s="4">
+        <v>40</v>
       </c>
       <c r="I4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="J4" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="K4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="L4" t="s" s="5">
-        <v>39</v>
+      <c r="J4" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="K4" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="L4" t="s" s="4">
+        <v>40</v>
       </c>
       <c r="M4" t="s" s="2">
         <v>38</v>
@@ -645,14 +645,14 @@
       <c r="R4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="S4" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="T4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="U4" t="s" s="5">
-        <v>39</v>
+      <c r="S4" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="T4" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="U4" t="s" s="4">
+        <v>40</v>
       </c>
       <c r="V4" t="s" s="2">
         <v>38</v>
@@ -672,14 +672,14 @@
       <c r="AA4" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="AB4" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="AC4" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AD4" t="s" s="5">
-        <v>39</v>
+      <c r="AB4" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="AC4" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="AD4" t="s" s="4">
+        <v>40</v>
       </c>
       <c r="AE4" t="s" s="2">
         <v>38</v>
@@ -808,26 +808,26 @@
       <c r="C6" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="D6" t="s" s="3">
+      <c r="D6" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="E6" t="s" s="5">
+        <v>39</v>
+      </c>
+      <c r="F6" t="s" s="3">
         <v>37</v>
       </c>
-      <c r="E6" t="s" s="1">
-        <v>35</v>
-      </c>
-      <c r="F6" t="s" s="4">
-        <v>40</v>
-      </c>
       <c r="G6" t="s" s="2">
         <v>38</v>
       </c>
       <c r="H6" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="I6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="J6" t="s" s="5">
-        <v>39</v>
+      <c r="I6" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="J6" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="K6" t="s" s="4">
         <v>40</v>
@@ -835,11 +835,11 @@
       <c r="L6" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="M6" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="N6" t="s" s="1">
-        <v>35</v>
+      <c r="M6" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="N6" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="O6" t="s" s="4">
         <v>40</v>
@@ -850,11 +850,11 @@
       <c r="Q6" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="R6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="S6" t="s" s="5">
-        <v>39</v>
+      <c r="R6" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="S6" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="T6" t="s" s="4">
         <v>40</v>
@@ -862,11 +862,11 @@
       <c r="U6" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="V6" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="W6" t="s" s="1">
-        <v>35</v>
+      <c r="V6" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="W6" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="X6" t="s" s="4">
         <v>40</v>
@@ -877,11 +877,11 @@
       <c r="Z6" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="AA6" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AB6" t="s" s="5">
-        <v>39</v>
+      <c r="AA6" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="AB6" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="AC6" t="s" s="4">
         <v>40</v>
@@ -889,11 +889,11 @@
       <c r="AD6" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="AE6" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="AF6" t="s" s="1">
-        <v>35</v>
+      <c r="AE6" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="AF6" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="AG6" t="s" s="0">
         <v>41</v>
@@ -1019,11 +1019,11 @@
       <c r="D8" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="E8" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="F8" t="s" s="5">
-        <v>39</v>
+      <c r="E8" t="s" s="3">
+        <v>37</v>
+      </c>
+      <c r="F8" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="G8" t="s" s="3">
         <v>37</v>
@@ -1031,11 +1031,11 @@
       <c r="H8" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="I8" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="J8" t="s" s="1">
-        <v>35</v>
+      <c r="I8" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="J8" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="K8" t="s" s="4">
         <v>40</v>
@@ -1046,11 +1046,11 @@
       <c r="M8" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="N8" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="O8" t="s" s="5">
-        <v>39</v>
+      <c r="N8" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="O8" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="P8" t="s" s="4">
         <v>40</v>
@@ -1058,11 +1058,11 @@
       <c r="Q8" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="R8" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="S8" t="s" s="1">
-        <v>35</v>
+      <c r="R8" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="S8" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="T8" t="s" s="4">
         <v>40</v>
@@ -1073,11 +1073,11 @@
       <c r="V8" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="W8" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="X8" t="s" s="5">
-        <v>39</v>
+      <c r="W8" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="X8" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="Y8" t="s" s="4">
         <v>40</v>
@@ -1085,11 +1085,11 @@
       <c r="Z8" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="AA8" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="AB8" t="s" s="1">
-        <v>35</v>
+      <c r="AA8" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="AB8" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="AC8" t="s" s="4">
         <v>40</v>
@@ -1100,8 +1100,8 @@
       <c r="AE8" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="AF8" t="s" s="2">
-        <v>38</v>
+      <c r="AF8" t="s" s="4">
+        <v>40</v>
       </c>
       <c r="AG8" t="s" s="0">
         <v>41</v>
@@ -1227,11 +1227,11 @@
       <c r="D10" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="E10" t="s" s="3">
-        <v>37</v>
-      </c>
-      <c r="F10" t="s" s="1">
-        <v>35</v>
+      <c r="E10" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="G10" t="s" s="4">
         <v>40</v>
@@ -1242,11 +1242,11 @@
       <c r="I10" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="J10" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="K10" t="s" s="5">
-        <v>39</v>
+      <c r="J10" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="K10" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="L10" t="s" s="4">
         <v>40</v>
@@ -1254,11 +1254,11 @@
       <c r="M10" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="N10" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="O10" t="s" s="1">
-        <v>35</v>
+      <c r="N10" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="O10" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="P10" t="s" s="4">
         <v>40</v>
@@ -1269,11 +1269,11 @@
       <c r="R10" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="S10" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="T10" t="s" s="5">
-        <v>39</v>
+      <c r="S10" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="T10" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="U10" t="s" s="4">
         <v>40</v>
@@ -1281,11 +1281,11 @@
       <c r="V10" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="W10" t="s" s="4">
-        <v>40</v>
-      </c>
-      <c r="X10" t="s" s="1">
-        <v>35</v>
+      <c r="W10" t="s" s="2">
+        <v>38</v>
+      </c>
+      <c r="X10" t="s" s="5">
+        <v>39</v>
       </c>
       <c r="Y10" t="s" s="4">
         <v>40</v>
@@ -1296,11 +1296,11 @@
       <c r="AA10" t="s" s="5">
         <v>39</v>
       </c>
-      <c r="AB10" t="s" s="2">
-        <v>38</v>
-      </c>
-      <c r="AC10" t="s" s="5">
-        <v>39</v>
+      <c r="AB10" t="s" s="4">
+        <v>40</v>
+      </c>
+      <c r="AC10" t="s" s="1">
+        <v>35</v>
       </c>
       <c r="AD10" t="s" s="4">
         <v>40</v>
@@ -1308,8 +1308,8 @@
       <c r="AE10" t="s" s="1">
         <v>35</v>
       </c>
-      <c r="AF10" t="s" s="4">
-        <v>40</v>
+      <c r="AF10" t="s" s="2">
+        <v>38</v>
       </c>
       <c r="AG10" t="s" s="0">
         <v>41</v>

</xml_diff>